<commit_message>
feat(laporan): opsi terakhir dan preset, filter pilih banyak, Excel data saja, ekspor daftar lewat antrean (K-24..K-29)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/apperp/management-aset/resources/laporan/laporan-pemusnahan-aset/standar.xlsx
+++ b/modules/apperp/management-aset/resources/laporan/laporan-pemusnahan-aset/standar.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="53">
   <si>
     <t>${kop.logo_kiri}</t>
   </si>
@@ -89,6 +89,18 @@
   </si>
   <si>
     <t>${jumlah_dokumen}</t>
+  </si>
+  <si>
+    <t>Lokasi</t>
+  </si>
+  <si>
+    <t>${filter_lokasi}</t>
+  </si>
+  <si>
+    <t>Kondisi</t>
+  </si>
+  <si>
+    <t>${filter_kondisi}</t>
   </si>
   <si>
     <t>No.</t>
@@ -717,79 +729,93 @@
         <v>23</v>
       </c>
     </row>
+    <row r="9" spans="1:11">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
     <row r="10" spans="1:11" customHeight="1" ht="32">
       <c r="A10" s="7" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E11" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F11" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G11" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="H11" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I11" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="J11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="K11" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="8" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -799,10 +825,10 @@
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="K12" s="8"/>
     </row>

</xml_diff>

<commit_message>
feat(laporan): opsi terakhir dan preset, filter pilih banyak, Excel data saja, ekspor daftar lewat antrean (K-24..K-29) (#223)
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/apperp/management-aset/resources/laporan/laporan-pemusnahan-aset/standar.xlsx
+++ b/modules/apperp/management-aset/resources/laporan/laporan-pemusnahan-aset/standar.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="53">
   <si>
     <t>${kop.logo_kiri}</t>
   </si>
@@ -89,6 +89,18 @@
   </si>
   <si>
     <t>${jumlah_dokumen}</t>
+  </si>
+  <si>
+    <t>Lokasi</t>
+  </si>
+  <si>
+    <t>${filter_lokasi}</t>
+  </si>
+  <si>
+    <t>Kondisi</t>
+  </si>
+  <si>
+    <t>${filter_kondisi}</t>
   </si>
   <si>
     <t>No.</t>
@@ -717,79 +729,93 @@
         <v>23</v>
       </c>
     </row>
+    <row r="9" spans="1:11">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
     <row r="10" spans="1:11" customHeight="1" ht="32">
       <c r="A10" s="7" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E11" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F11" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G11" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="H11" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I11" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="J11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="K11" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="8" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -799,10 +825,10 @@
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="K12" s="8"/>
     </row>

</xml_diff>